<commit_message>
Modiche alla presentazione per la tesi
</commit_message>
<xml_diff>
--- a/Presentazione/tempi_presentazione.xlsx
+++ b/Presentazione/tempi_presentazione.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Marco\Desktop\Tesi Bella\Tesi-Magistrale---M.-Mecarelli-F.-Santini\Presentazione\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6645A44B-1FB4-4C26-A05A-FCC06805D962}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2F9CDA39-304A-4BEA-B969-1226ED070AF2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="12000" yWindow="5970" windowWidth="12000" windowHeight="6930" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="12000" windowHeight="12900" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Foglio1" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="31">
   <si>
     <t>minuti</t>
   </si>
@@ -88,13 +88,52 @@
   </si>
   <si>
     <t>Test</t>
+  </si>
+  <si>
+    <t>OLD TESI BELLA V1</t>
+  </si>
+  <si>
+    <t>OLD TESI BELLA V2</t>
+  </si>
+  <si>
+    <t>Introduzione</t>
+  </si>
+  <si>
+    <t>Timing Covert Channel</t>
+  </si>
+  <si>
+    <t>Storage Covert Channel</t>
+  </si>
+  <si>
+    <t>Behavioural Covert Channel</t>
+  </si>
+  <si>
+    <t>Test e Risultati</t>
+  </si>
+  <si>
+    <t>Conclusioni</t>
+  </si>
+  <si>
+    <t>Comunicazione Inizializzazione</t>
+  </si>
+  <si>
+    <t>Comunicazione Impostazione</t>
+  </si>
+  <si>
+    <t>Comunicazione Comunicazione</t>
+  </si>
+  <si>
+    <t>Comunicazione Chiusura</t>
+  </si>
+  <si>
+    <t>Comunicazione Introduzione</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -110,13 +149,33 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF92D050"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -131,9 +190,15 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normale" xfId="0" builtinId="0"/>
@@ -414,40 +479,29 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F15"/>
+  <dimension ref="A1:I35"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-      <c r="E1" t="s">
+      <c r="A1" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="B1" s="2"/>
+      <c r="C1" s="2"/>
+      <c r="D1" s="2"/>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" t="s">
+        <v>1</v>
+      </c>
+      <c r="E2" t="s">
         <v>3</v>
       </c>
-      <c r="F1" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A2">
-        <v>0</v>
-      </c>
-      <c r="B2">
-        <v>48</v>
-      </c>
-      <c r="C2" t="s">
-        <v>4</v>
-      </c>
-      <c r="E2">
-        <f>SUM(B:B)</f>
-        <v>449</v>
-      </c>
-      <c r="F2" s="1">
-        <f>SUM(A:A)+E3</f>
-        <v>30</v>
+      <c r="F2" t="s">
+        <v>2</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
@@ -455,36 +509,44 @@
         <v>0</v>
       </c>
       <c r="B3">
-        <v>31</v>
+        <v>48</v>
       </c>
       <c r="C3" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E3">
-        <f>_xlfn.FLOOR.MATH(SUM(B:B)/60)</f>
-        <v>7</v>
+        <f>SUM($B3:$B16)</f>
+        <v>449</v>
+      </c>
+      <c r="F3" s="1">
+        <f>SUM($A3:$A16)+$E4</f>
+        <v>30</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B4">
-        <v>0</v>
+        <v>31</v>
       </c>
       <c r="C4" t="s">
-        <v>15</v>
+        <v>5</v>
+      </c>
+      <c r="E4">
+        <f>_xlfn.FLOOR.MATH(E3/60)</f>
+        <v>7</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B5">
-        <v>49</v>
+        <v>0</v>
       </c>
       <c r="C5" t="s">
-        <v>6</v>
+        <v>15</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
@@ -492,21 +554,21 @@
         <v>0</v>
       </c>
       <c r="B6">
-        <v>0</v>
+        <v>49</v>
       </c>
       <c r="C6" t="s">
-        <v>12</v>
+        <v>6</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B7">
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="C7" t="s">
-        <v>8</v>
+        <v>12</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
@@ -514,10 +576,10 @@
         <v>1</v>
       </c>
       <c r="B8">
-        <v>35</v>
+        <v>20</v>
       </c>
       <c r="C8" t="s">
-        <v>16</v>
+        <v>8</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
@@ -525,79 +587,299 @@
         <v>1</v>
       </c>
       <c r="B9">
-        <v>12</v>
+        <v>35</v>
       </c>
       <c r="C9" t="s">
-        <v>9</v>
+        <v>16</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B10">
-        <v>55</v>
+        <v>12</v>
       </c>
       <c r="C10" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="B11">
         <v>55</v>
       </c>
       <c r="C11" t="s">
-        <v>10</v>
+        <v>7</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="B12">
-        <v>22</v>
+        <v>55</v>
       </c>
       <c r="C12" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="B13">
-        <v>56</v>
+        <v>22</v>
       </c>
       <c r="C13" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A14">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="B14">
-        <v>16</v>
+        <v>56</v>
       </c>
       <c r="C14" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="B15">
+        <v>16</v>
+      </c>
+      <c r="C15" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A16">
+        <v>2</v>
+      </c>
+      <c r="B16">
         <v>50</v>
       </c>
-      <c r="C15" t="s">
+      <c r="C16" t="s">
         <v>14</v>
       </c>
     </row>
+    <row r="18" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A18" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="B18" s="2"/>
+      <c r="C18" s="2"/>
+      <c r="D18" s="2"/>
+    </row>
+    <row r="19" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>0</v>
+      </c>
+      <c r="B19" t="s">
+        <v>1</v>
+      </c>
+      <c r="F19" t="s">
+        <v>3</v>
+      </c>
+      <c r="G19" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="20" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="B20">
+        <v>30</v>
+      </c>
+      <c r="C20" t="s">
+        <v>20</v>
+      </c>
+      <c r="F20">
+        <f>SUM($B20:$B33)</f>
+        <v>363</v>
+      </c>
+      <c r="G20" s="1">
+        <f>SUM($A20:$A33)+$F21</f>
+        <v>17</v>
+      </c>
+      <c r="I20" s="4">
+        <f>_xlfn.CEILING.MATH(SUM($B20:$B22)/60)+SUM($A20:$A22)</f>
+        <v>2</v>
+      </c>
+    </row>
+    <row r="21" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="B21">
+        <v>16</v>
+      </c>
+      <c r="D21" t="s">
+        <v>5</v>
+      </c>
+      <c r="F21">
+        <f>_xlfn.CEILING.MATH(F20/60)</f>
+        <v>7</v>
+      </c>
+      <c r="I21" s="4"/>
+    </row>
+    <row r="22" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A22">
+        <v>1</v>
+      </c>
+      <c r="B22">
+        <v>2</v>
+      </c>
+      <c r="D22" t="s">
+        <v>15</v>
+      </c>
+      <c r="I22" s="4"/>
+    </row>
+    <row r="23" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="I23" s="3">
+        <f>_xlfn.CEILING.MATH(SUM($B23:$B28)/60)+SUM($A23:$A28)</f>
+        <v>4</v>
+      </c>
+    </row>
+    <row r="24" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="B24">
+        <v>23</v>
+      </c>
+      <c r="D24" t="s">
+        <v>30</v>
+      </c>
+      <c r="I24" s="3"/>
+    </row>
+    <row r="25" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="B25">
+        <v>46</v>
+      </c>
+      <c r="D25" t="s">
+        <v>26</v>
+      </c>
+      <c r="I25" s="3"/>
+    </row>
+    <row r="26" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A26">
+        <v>1</v>
+      </c>
+      <c r="B26">
+        <v>6</v>
+      </c>
+      <c r="D26" t="s">
+        <v>27</v>
+      </c>
+      <c r="I26" s="3"/>
+    </row>
+    <row r="27" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A27">
+        <v>0</v>
+      </c>
+      <c r="B27">
+        <v>57</v>
+      </c>
+      <c r="D27" t="s">
+        <v>28</v>
+      </c>
+      <c r="I27" s="3"/>
+    </row>
+    <row r="28" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="B28">
+        <v>18</v>
+      </c>
+      <c r="D28" t="s">
+        <v>29</v>
+      </c>
+      <c r="I28" s="3"/>
+    </row>
+    <row r="29" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A29">
+        <v>2</v>
+      </c>
+      <c r="B29">
+        <v>53</v>
+      </c>
+      <c r="C29" t="s">
+        <v>21</v>
+      </c>
+      <c r="I29" s="5">
+        <f>_xlfn.CEILING.MATH(SUM($B29)/60)+SUM($A29)</f>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="30" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A30">
+        <v>2</v>
+      </c>
+      <c r="B30">
+        <v>4</v>
+      </c>
+      <c r="C30" t="s">
+        <v>22</v>
+      </c>
+      <c r="I30" s="5">
+        <f t="shared" ref="I30:I33" si="0">_xlfn.CEILING.MATH(SUM($B30)/60)+SUM($A30)</f>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="31" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A31">
+        <v>1</v>
+      </c>
+      <c r="B31">
+        <v>12</v>
+      </c>
+      <c r="C31" t="s">
+        <v>23</v>
+      </c>
+      <c r="I31" s="5">
+        <f t="shared" si="0"/>
+        <v>2</v>
+      </c>
+    </row>
+    <row r="32" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A32">
+        <v>2</v>
+      </c>
+      <c r="B32">
+        <v>46</v>
+      </c>
+      <c r="C32" t="s">
+        <v>24</v>
+      </c>
+      <c r="I32" s="5">
+        <f t="shared" si="0"/>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="33" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A33">
+        <v>1</v>
+      </c>
+      <c r="B33">
+        <v>50</v>
+      </c>
+      <c r="C33" t="s">
+        <v>25</v>
+      </c>
+      <c r="I33" s="5">
+        <f t="shared" si="0"/>
+        <v>2</v>
+      </c>
+    </row>
+    <row r="35" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="I35">
+        <f>SUM(I20:I33)</f>
+        <v>19</v>
+      </c>
+    </row>
   </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A18:D18"/>
+  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Push dei file della presentazione
</commit_message>
<xml_diff>
--- a/Presentazione/tempi_presentazione.xlsx
+++ b/Presentazione/tempi_presentazione.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Marco\Desktop\Tesi Bella\Tesi-Magistrale---M.-Mecarelli-F.-Santini\Presentazione\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2F9CDA39-304A-4BEA-B969-1226ED070AF2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ABB53E6D-8C71-4C3B-A958-FF00903F8273}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="12000" windowHeight="12900" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="12000" yWindow="0" windowWidth="12000" windowHeight="12900" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Foglio1" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="30">
   <si>
     <t>minuti</t>
   </si>
@@ -93,9 +93,6 @@
     <t>OLD TESI BELLA V1</t>
   </si>
   <si>
-    <t>OLD TESI BELLA V2</t>
-  </si>
-  <si>
     <t>Introduzione</t>
   </si>
   <si>
@@ -111,22 +108,22 @@
     <t>Test e Risultati</t>
   </si>
   <si>
-    <t>Conclusioni</t>
-  </si>
-  <si>
-    <t>Comunicazione Inizializzazione</t>
-  </si>
-  <si>
-    <t>Comunicazione Impostazione</t>
-  </si>
-  <si>
-    <t>Comunicazione Comunicazione</t>
-  </si>
-  <si>
-    <t>Comunicazione Chiusura</t>
-  </si>
-  <si>
-    <t>Comunicazione Introduzione</t>
+    <t>6:44.71</t>
+  </si>
+  <si>
+    <t>Introi+Imple</t>
+  </si>
+  <si>
+    <t>Covert</t>
+  </si>
+  <si>
+    <t>Totale</t>
+  </si>
+  <si>
+    <t>Implementazione</t>
+  </si>
+  <si>
+    <t>TESI BELLA V2</t>
   </si>
 </sst>
 </file>
@@ -158,7 +155,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -168,12 +165,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFFF00"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FF92D050"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -190,14 +181,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -479,16 +469,16 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:I35"/>
+  <dimension ref="A1:P35"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A1" s="2" t="s">
+      <c r="A1" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="B1" s="2"/>
-      <c r="C1" s="2"/>
-      <c r="D1" s="2"/>
+      <c r="B1" s="3"/>
+      <c r="C1" s="3"/>
+      <c r="D1" s="3"/>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
@@ -670,15 +660,15 @@
         <v>14</v>
       </c>
     </row>
-    <row r="18" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A18" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="B18" s="2"/>
-      <c r="C18" s="2"/>
-      <c r="D18" s="2"/>
-    </row>
-    <row r="19" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A18" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="B18" s="3"/>
+      <c r="C18" s="3"/>
+      <c r="D18" s="3"/>
+    </row>
+    <row r="19" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>0</v>
       </c>
@@ -692,188 +682,177 @@
         <v>2</v>
       </c>
     </row>
-    <row r="20" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A20">
+        <v>1</v>
+      </c>
       <c r="B20">
-        <v>30</v>
+        <v>45</v>
       </c>
       <c r="C20" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F20">
         <f>SUM($B20:$B33)</f>
-        <v>363</v>
+        <v>261</v>
       </c>
       <c r="G20" s="1">
-        <f>SUM($A20:$A33)+$F21</f>
-        <v>17</v>
-      </c>
-      <c r="I20" s="4">
-        <f>_xlfn.CEILING.MATH(SUM($B20:$B22)/60)+SUM($A20:$A22)</f>
+        <f>SUM($A20:$A29)+$F22</f>
+        <v>15.35</v>
+      </c>
+      <c r="I20" s="4"/>
+    </row>
+    <row r="21" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A21">
         <v>2</v>
       </c>
-    </row>
-    <row r="21" spans="1:9" x14ac:dyDescent="0.25">
       <c r="B21">
-        <v>16</v>
-      </c>
-      <c r="D21" t="s">
         <v>5</v>
+      </c>
+      <c r="C21" t="s">
+        <v>28</v>
       </c>
       <c r="F21">
         <f>_xlfn.CEILING.MATH(F20/60)</f>
+        <v>5</v>
+      </c>
+      <c r="I21" s="4"/>
+    </row>
+    <row r="22" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A22">
+        <v>1</v>
+      </c>
+      <c r="B22">
+        <v>19</v>
+      </c>
+      <c r="C22" t="s">
+        <v>8</v>
+      </c>
+      <c r="F22">
+        <f>F20/60</f>
+        <v>4.3499999999999996</v>
+      </c>
+      <c r="I22" s="4"/>
+      <c r="M22" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="23" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="B23">
+        <v>31</v>
+      </c>
+      <c r="C23" t="s">
+        <v>16</v>
+      </c>
+      <c r="I23" s="4"/>
+      <c r="N23" t="s">
+        <v>25</v>
+      </c>
+      <c r="O23" s="2">
         <v>7</v>
       </c>
-      <c r="I21" s="4"/>
-    </row>
-    <row r="22" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A22">
-        <v>1</v>
-      </c>
-      <c r="B22">
+      <c r="P23">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="24" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="B24">
+        <v>38</v>
+      </c>
+      <c r="C24" t="s">
+        <v>9</v>
+      </c>
+      <c r="I24" s="4"/>
+      <c r="N24" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="25" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A25">
         <v>2</v>
       </c>
-      <c r="D22" t="s">
-        <v>15</v>
-      </c>
-      <c r="I22" s="4"/>
-    </row>
-    <row r="23" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="I23" s="3">
-        <f>_xlfn.CEILING.MATH(SUM($B23:$B28)/60)+SUM($A23:$A28)</f>
-        <v>4</v>
-      </c>
-    </row>
-    <row r="24" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="B24">
+      <c r="B25">
+        <v>11</v>
+      </c>
+      <c r="C25" t="s">
+        <v>20</v>
+      </c>
+      <c r="I25" s="4"/>
+      <c r="N25" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="26" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A26">
+        <v>2</v>
+      </c>
+      <c r="B26">
+        <v>52</v>
+      </c>
+      <c r="C26" t="s">
+        <v>21</v>
+      </c>
+      <c r="I26" s="4"/>
+      <c r="O26" s="2">
+        <f>SUM(O23:O25)</f>
+        <v>7</v>
+      </c>
+      <c r="P26" s="2">
+        <f>SUM(P23:P25)</f>
+        <v>50</v>
+      </c>
+    </row>
+    <row r="27" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A27">
+        <v>1</v>
+      </c>
+      <c r="B27">
+        <v>6</v>
+      </c>
+      <c r="C27" t="s">
+        <v>22</v>
+      </c>
+      <c r="I27" s="4"/>
+      <c r="N27" t="s">
+        <v>27</v>
+      </c>
+      <c r="O27" s="2">
+        <f>O26+_xlfn.CEILING.MATH(P26/60)</f>
+        <v>8</v>
+      </c>
+    </row>
+    <row r="28" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A28">
+        <v>2</v>
+      </c>
+      <c r="B28">
+        <v>54</v>
+      </c>
+      <c r="C28" t="s">
         <v>23</v>
       </c>
-      <c r="D24" t="s">
-        <v>30</v>
-      </c>
-      <c r="I24" s="3"/>
-    </row>
-    <row r="25" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="B25">
-        <v>46</v>
-      </c>
-      <c r="D25" t="s">
-        <v>26</v>
-      </c>
-      <c r="I25" s="3"/>
-    </row>
-    <row r="26" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A26">
-        <v>1</v>
-      </c>
-      <c r="B26">
-        <v>6</v>
-      </c>
-      <c r="D26" t="s">
-        <v>27</v>
-      </c>
-      <c r="I26" s="3"/>
-    </row>
-    <row r="27" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A27">
-        <v>0</v>
-      </c>
-      <c r="B27">
-        <v>57</v>
-      </c>
-      <c r="D27" t="s">
-        <v>28</v>
-      </c>
-      <c r="I27" s="3"/>
-    </row>
-    <row r="28" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="B28">
-        <v>18</v>
-      </c>
-      <c r="D28" t="s">
-        <v>29</v>
-      </c>
-      <c r="I28" s="3"/>
-    </row>
-    <row r="29" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A29">
-        <v>2</v>
-      </c>
-      <c r="B29">
-        <v>53</v>
-      </c>
-      <c r="C29" t="s">
-        <v>21</v>
-      </c>
-      <c r="I29" s="5">
-        <f>_xlfn.CEILING.MATH(SUM($B29)/60)+SUM($A29)</f>
-        <v>3</v>
-      </c>
-    </row>
-    <row r="30" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A30">
-        <v>2</v>
-      </c>
-      <c r="B30">
-        <v>4</v>
-      </c>
-      <c r="C30" t="s">
-        <v>22</v>
-      </c>
-      <c r="I30" s="5">
-        <f t="shared" ref="I30:I33" si="0">_xlfn.CEILING.MATH(SUM($B30)/60)+SUM($A30)</f>
-        <v>3</v>
-      </c>
-    </row>
-    <row r="31" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A31">
-        <v>1</v>
-      </c>
-      <c r="B31">
-        <v>12</v>
-      </c>
-      <c r="C31" t="s">
-        <v>23</v>
-      </c>
-      <c r="I31" s="5">
-        <f t="shared" si="0"/>
-        <v>2</v>
-      </c>
-    </row>
-    <row r="32" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A32">
-        <v>2</v>
-      </c>
-      <c r="B32">
-        <v>46</v>
-      </c>
-      <c r="C32" t="s">
-        <v>24</v>
-      </c>
-      <c r="I32" s="5">
-        <f t="shared" si="0"/>
-        <v>3</v>
-      </c>
-    </row>
-    <row r="33" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A33">
-        <v>1</v>
-      </c>
-      <c r="B33">
-        <v>50</v>
-      </c>
-      <c r="C33" t="s">
-        <v>25</v>
-      </c>
-      <c r="I33" s="5">
-        <f t="shared" si="0"/>
-        <v>2</v>
-      </c>
-    </row>
-    <row r="35" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="I35">
-        <f>SUM(I20:I33)</f>
-        <v>19</v>
-      </c>
+      <c r="I28" s="4"/>
+    </row>
+    <row r="29" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="I29" s="4"/>
+    </row>
+    <row r="30" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="I30" s="4"/>
+    </row>
+    <row r="31" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="I31" s="4"/>
+    </row>
+    <row r="32" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="I32" s="4"/>
+    </row>
+    <row r="33" spans="9:9" x14ac:dyDescent="0.25">
+      <c r="I33" s="4"/>
+    </row>
+    <row r="34" spans="9:9" x14ac:dyDescent="0.25">
+      <c r="I34" s="4"/>
+    </row>
+    <row r="35" spans="9:9" x14ac:dyDescent="0.25">
+      <c r="I35" s="4"/>
     </row>
   </sheetData>
   <mergeCells count="2">

</xml_diff>